<commit_message>
Bao[spec](bookImport): update import template to generate 2 copies per book
</commit_message>
<xml_diff>
--- a/database/supabase/templates/template_import_books.xlsx
+++ b/database/supabase/templates/template_import_books.xlsx
@@ -1468,7 +1468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1530,17 +1530,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>9780134685991</t>
+          <t>9780132350884</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>BC9780134685991-03</t>
+          <t>BC9780132350884-01</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-5991-3</t>
+          <t>Kệ CS-0884-1</t>
         </is>
       </c>
     </row>
@@ -1552,1219 +1552,794 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>BC9780132350884-01</t>
+          <t>BC9780132350884-02</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-0884-1</t>
+          <t>Kệ CS-0884-2</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>9780132350884</t>
+          <t>9780201633610</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>BC9780132350884-02</t>
+          <t>BC9780201633610-01</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-0884-2</t>
+          <t>Kệ CS-3610-1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>9780132350884</t>
+          <t>9780201633610</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>BC9780132350884-03</t>
+          <t>BC9780201633610-02</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-0884-3</t>
+          <t>Kệ CS-3610-2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>9780201633610</t>
+          <t>9781119560822</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BC9780201633610-01</t>
+          <t>BC9781119560822-01</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-3610-1</t>
+          <t>Kệ GEN-0822-1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>9780201633610</t>
+          <t>9781119560822</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>BC9780201633610-02</t>
+          <t>BC9781119560822-02</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-3610-2</t>
+          <t>Kệ GEN-0822-2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>9780201633610</t>
+          <t>9780321356680</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>BC9780201633610-03</t>
+          <t>BC9780321356680-01</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-3610-3</t>
+          <t>Kệ CS-6680-1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>9781119560822</t>
+          <t>9780321356680</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>BC9781119560822-01</t>
+          <t>BC9780321356680-02</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-0822-1</t>
+          <t>Kệ CS-6680-2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>9781119560822</t>
+          <t>9780073523323</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>BC9781119560822-02</t>
+          <t>BC9780073523323-01</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-0822-2</t>
+          <t>Kệ GEN-3323-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>9781119560822</t>
+          <t>9780073523323</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>BC9781119560822-03</t>
+          <t>BC9780073523323-02</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-0822-3</t>
+          <t>Kệ GEN-3323-2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>9780321356680</t>
+          <t>9780199232741</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>BC9780321356680-01</t>
+          <t>BC9780199232741-01</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-6680-1</t>
+          <t>Kệ GEN-2741-1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>9780321356680</t>
+          <t>9780199232741</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>BC9780321356680-02</t>
+          <t>BC9780199232741-02</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-6680-2</t>
+          <t>Kệ GEN-2741-2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>9780321356680</t>
+          <t>9781449331818</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>BC9780321356680-03</t>
+          <t>BC9781449331818-01</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-6680-3</t>
+          <t>Kệ CS-1818-1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>9780073523323</t>
+          <t>9781449331818</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>BC9780073523323-01</t>
+          <t>BC9781449331818-02</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3323-1</t>
+          <t>Kệ CS-1818-2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>9780073523323</t>
+          <t>9780132145374</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>BC9780073523323-02</t>
+          <t>BC9780132145374-01</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3323-2</t>
+          <t>Kệ CS-5374-1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>9780073523323</t>
+          <t>9780132145374</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>BC9780073523323-03</t>
+          <t>BC9780132145374-02</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3323-3</t>
+          <t>Kệ CS-5374-2</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>9780199232741</t>
+          <t>9780321573513</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>BC9780199232741-01</t>
+          <t>BC9780321573513-01</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-2741-1</t>
+          <t>Kệ GEN-3513-1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>9780199232741</t>
+          <t>9780321573513</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>BC9780199232741-02</t>
+          <t>BC9780321573513-02</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-2741-2</t>
+          <t>Kệ GEN-3513-2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>9780199232741</t>
+          <t>9780134093413</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>BC9780199232741-03</t>
+          <t>BC9780134093413-01</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-2741-3</t>
+          <t>Kệ GEN-3413-1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>9781449331818</t>
+          <t>9780134093413</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>BC9781449331818-01</t>
+          <t>BC9780134093413-02</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-1818-1</t>
+          <t>Kệ GEN-3413-2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>9781449331818</t>
+          <t>9780470503201</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>BC9781449331818-02</t>
+          <t>BC9780470503201-01</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-1818-2</t>
+          <t>Kệ GEN-3201-1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>9781449331818</t>
+          <t>9780470503201</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>BC9781449331818-03</t>
+          <t>BC9780470503201-02</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-1818-3</t>
+          <t>Kệ GEN-3201-2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>9780132145374</t>
+          <t>9780078021558</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>BC9780132145374-01</t>
+          <t>BC9780078021558-01</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-5374-1</t>
+          <t>Kệ GEN-1558-1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>9780132145374</t>
+          <t>9780078021558</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>BC9780132145374-02</t>
+          <t>BC9780078021558-02</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-5374-2</t>
+          <t>Kệ GEN-1558-2</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>9780132145374</t>
+          <t>9780136006633</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>BC9780132145374-03</t>
+          <t>BC9780136006633-01</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Kệ CS-5374-3</t>
+          <t>Kệ GEN-6633-1</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>9780321573513</t>
+          <t>9780136006633</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>BC9780321573513-01</t>
+          <t>BC9780136006633-02</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3513-1</t>
+          <t>Kệ GEN-6633-2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>9780321573513</t>
+          <t>9780470646151</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>BC9780321573513-02</t>
+          <t>BC9780470646151-01</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3513-2</t>
+          <t>Kệ GEN-6151-1</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>9780321573513</t>
+          <t>9780470646151</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>BC9780321573513-03</t>
+          <t>BC9780470646151-02</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3513-3</t>
+          <t>Kệ GEN-6151-2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>9780134093413</t>
+          <t>9781285057903</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>BC9780134093413-01</t>
+          <t>BC9781285057903-01</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3413-1</t>
+          <t>Kệ GEN-7903-1</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>9780134093413</t>
+          <t>9781285057903</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>BC9780134093413-02</t>
+          <t>BC9781285057903-02</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3413-2</t>
+          <t>Kệ GEN-7903-2</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>9780134093413</t>
+          <t>9780133098754</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>BC9780134093413-03</t>
+          <t>BC9780133098754-01</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3413-3</t>
+          <t>Kệ GEN-8754-1</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>9780470503201</t>
+          <t>9780133098754</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>BC9780470503201-01</t>
+          <t>BC9780133098754-02</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3201-1</t>
+          <t>Kệ GEN-8754-2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>9780470503201</t>
+          <t>9781133312789</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>BC9780470503201-02</t>
+          <t>BC9781133312789-01</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3201-2</t>
+          <t>Kệ GEN-2789-1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>9780470503201</t>
+          <t>9781133312789</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>BC9780470503201-03</t>
+          <t>BC9781133312789-02</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-3201-3</t>
+          <t>Kệ GEN-2789-2</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>9780078021558</t>
+          <t>9780199571123</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>BC9780078021558-01</t>
+          <t>BC9780199571123-01</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-1558-1</t>
+          <t>Kệ GEN-1123-1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>9780078021558</t>
+          <t>9780199571123</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>BC9780078021558-02</t>
+          <t>BC9780199571123-02</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-1558-2</t>
+          <t>Kệ GEN-1123-2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>9780078021558</t>
+          <t>9781305073036</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>BC9780078021558-03</t>
+          <t>BC9781305073036-01</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-1558-3</t>
+          <t>Kệ GEN-3036-1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>9780136006633</t>
+          <t>9781305073036</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>BC9780136006633-01</t>
+          <t>BC9781305073036-02</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-6633-1</t>
+          <t>Kệ GEN-3036-2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>9780136006633</t>
+          <t>9780321838964</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>BC9780136006633-02</t>
+          <t>BC9780321838964-01</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-6633-2</t>
+          <t>Kệ CS-8964-1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>9780136006633</t>
+          <t>9780321838964</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>BC9780136006633-03</t>
+          <t>BC9780321838964-02</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-6633-3</t>
+          <t>Kệ CS-8964-2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>9780470646151</t>
+          <t>9780133914641</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>BC9780470646151-01</t>
+          <t>BC9780133914641-01</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-6151-1</t>
+          <t>Kệ CS-4641-1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>9780470646151</t>
+          <t>9780133914641</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>BC9780470646151-02</t>
+          <t>BC9780133914641-02</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-6151-2</t>
+          <t>Kệ CS-4641-2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>9780470646151</t>
+          <t>9781491950296</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>BC9780470646151-03</t>
+          <t>BC9781491950296-01</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-6151-3</t>
+          <t>Kệ CS-0296-1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>9781285057903</t>
+          <t>9781491950296</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>BC9781285057903-01</t>
+          <t>BC9781491950296-02</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-7903-1</t>
+          <t>Kệ CS-0296-2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>9781285057903</t>
+          <t>9781501257285</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>BC9781285057903-02</t>
+          <t>BC9781501257285-01</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-7903-2</t>
+          <t>Kệ GEN-7285-1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>9781285057903</t>
+          <t>9781501257285</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>BC9781285057903-03</t>
+          <t>BC9781501257285-02</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-7903-3</t>
+          <t>Kệ GEN-7285-2</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>9780133098754</t>
+          <t>9780073523859</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>BC9780133098754-01</t>
+          <t>BC9780073523859-01</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-8754-1</t>
+          <t>Kệ CS-3859-1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>9780133098754</t>
+          <t>9780073523859</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>BC9780133098754-02</t>
+          <t>BC9780073523859-02</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-8754-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>9780133098754</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>BC9780133098754-03</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-8754-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>9781133312789</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>BC9781133312789-01</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-2789-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>9781133312789</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>BC9781133312789-02</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-2789-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>9781133312789</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>BC9781133312789-03</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-2789-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>9780199571123</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>BC9780199571123-01</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-1123-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>9780199571123</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>BC9780199571123-02</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-1123-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>9780199571123</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>BC9780199571123-03</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-1123-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>9781305073036</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>BC9781305073036-01</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-3036-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>9781305073036</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>BC9781305073036-02</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-3036-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>9781305073036</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>BC9781305073036-03</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-3036-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>9780321838964</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>BC9780321838964-01</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-8964-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>9780321838964</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>BC9780321838964-02</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-8964-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>9780321838964</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>BC9780321838964-03</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-8964-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>9780133914641</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>BC9780133914641-01</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-4641-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>9780133914641</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>BC9780133914641-02</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-4641-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>9780133914641</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>BC9780133914641-03</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-4641-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>9781491950296</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>BC9781491950296-01</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-0296-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>9781491950296</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>BC9781491950296-02</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-0296-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>9781491950296</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>BC9781491950296-03</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-0296-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>9781501257285</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>BC9781501257285-01</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-7285-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>9781501257285</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>BC9781501257285-02</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-7285-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>9781501257285</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>BC9781501257285-03</t>
-        </is>
-      </c>
-      <c r="C73" s="3" t="inlineStr">
-        <is>
-          <t>Kệ GEN-7285-3</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>9780073523859</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>BC9780073523859-01</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-3859-1</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>9780073523859</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>BC9780073523859-02</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
           <t>Kệ CS-3859-2</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>9780073523859</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>BC9780073523859-03</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>Kệ CS-3859-3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bao[spec](bookImport): fix separator to semicolon and remove thousand separator format to resolve import error
</commit_message>
<xml_diff>
--- a/database/supabase/templates/template_import_books.xlsx
+++ b/database/supabase/templates/template_import_books.xlsx
@@ -84,7 +84,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -541,7 +541,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Coding,Reference</t>
+          <t>Textbook;Coding;Reference</t>
         </is>
       </c>
     </row>
@@ -579,7 +579,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Coding</t>
+          <t>Textbook;Coding</t>
         </is>
       </c>
     </row>
@@ -617,7 +617,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Reference,Theoretical</t>
+          <t>Reference;Theoretical</t>
         </is>
       </c>
     </row>
@@ -655,7 +655,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>Textbook,CaseStudy</t>
+          <t>Textbook;CaseStudy</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Coding,Theoretical</t>
+          <t>Textbook;Coding;Theoretical</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Theoretical</t>
+          <t>Textbook;Theoretical</t>
         </is>
       </c>
     </row>
@@ -769,7 +769,7 @@
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Introduction,Textbook</t>
+          <t>Introduction;Textbook</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>Reference,Advanced</t>
+          <t>Reference;Advanced</t>
         </is>
       </c>
     </row>
@@ -845,7 +845,7 @@
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>Textbook,AI_Driven,Advanced</t>
+          <t>Textbook;AI_Driven;Advanced</t>
         </is>
       </c>
     </row>
@@ -883,7 +883,7 @@
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Theoretical</t>
+          <t>Textbook;Theoretical</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Reference</t>
+          <t>Textbook;Reference</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>Introduction,Textbook</t>
+          <t>Introduction;Textbook</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Experimental</t>
+          <t>Textbook;Experimental</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>Biology &amp; Ecology,Medicine &amp; Health Sciences</t>
+          <t>Biology &amp; Ecology;Medicine &amp; Health Sciences</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>Textbook,LabManual</t>
+          <t>Textbook;LabManual</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Reference</t>
+          <t>Textbook;Reference</t>
         </is>
       </c>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>Introduction,Textbook</t>
+          <t>Introduction;Textbook</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>Textbook,CaseStudy,Strategic</t>
+          <t>Textbook;CaseStudy;Strategic</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>Chemistry,Pharmacy &amp; Biochemistry</t>
+          <t>Chemistry;Pharmacy &amp; Biochemistry</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>Textbook,LabManual</t>
+          <t>Textbook;LabManual</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>Introduction,Textbook</t>
+          <t>Introduction;Textbook</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Behavioral</t>
+          <t>Textbook;Behavioral</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Computer Science,Arts &amp; Design</t>
+          <t>Computer Science;Arts &amp; Design</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>Reference,Visual_Design</t>
+          <t>Reference;Visual_Design</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Management</t>
+          <t>Textbook;Management</t>
         </is>
       </c>
     </row>
@@ -1377,7 +1377,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>Reference,Advanced</t>
+          <t>Reference;Advanced</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>Reference,Management</t>
+          <t>Reference;Management</t>
         </is>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>Textbook,Theoretical,Advanced</t>
+          <t>Textbook;Theoretical;Advanced</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bao[feat]: update BookSearchServlet and book-search.jsp with improved search filters, seed data and test updates
</commit_message>
<xml_diff>
--- a/database/supabase/templates/template_import_books.xlsx
+++ b/database/supabase/templates/template_import_books.xlsx
@@ -532,7 +532,7 @@
         <v>2018</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>850000</v>
+        <v>125000</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -570,7 +570,7 @@
         <v>2008</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>650000</v>
+        <v>110000</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -608,7 +608,7 @@
         <v>1994</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>950000</v>
+        <v>135000</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -624,7 +624,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>9781119560822</t>
+          <t>9781119560821</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -646,7 +646,7 @@
         <v>2019</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>1200000</v>
+        <v>140000</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
@@ -684,7 +684,7 @@
         <v>2011</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>900000</v>
+        <v>130000</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
@@ -722,7 +722,7 @@
         <v>2015</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>800000</v>
+        <v>115000</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
         <v>2016</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>550000</v>
+        <v>85000</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
         <v>2017</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>1100000</v>
+        <v>145000</v>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
@@ -836,7 +836,7 @@
         <v>2010</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1500000</v>
+        <v>150000</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
         <v>2012</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>750000</v>
+        <v>105000</v>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
         <v>2016</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1600000</v>
+        <v>148000</v>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
         <v>2012</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>700000</v>
+        <v>95000</v>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
@@ -988,7 +988,7 @@
         <v>2013</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1300000</v>
+        <v>138000</v>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
@@ -1026,7 +1026,7 @@
         <v>2009</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>1420000</v>
+        <v>142000</v>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
@@ -1064,7 +1064,7 @@
         <v>2011</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>1800000</v>
+        <v>150000</v>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         <v>2013</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>600000</v>
+        <v>75000</v>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
         <v>2015</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>1150000</v>
+        <v>120000</v>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
@@ -1178,7 +1178,7 @@
         <v>2015</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>980000</v>
+        <v>118000</v>
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
@@ -1216,7 +1216,7 @@
         <v>2014</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>670000</v>
+        <v>88000</v>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
@@ -1254,7 +1254,7 @@
         <v>2015</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>850000</v>
+        <v>98000</v>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
@@ -1292,7 +1292,7 @@
         <v>2016</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>930000</v>
+        <v>128000</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
         <v>2015</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>950000</v>
+        <v>132000</v>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
@@ -1368,7 +1368,7 @@
         <v>2017</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>650000</v>
+        <v>92000</v>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
@@ -1406,7 +1406,7 @@
         <v>2014</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>450000</v>
+        <v>65000</v>
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
@@ -1444,7 +1444,7 @@
         <v>2009</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>1400000</v>
+        <v>145000</v>
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
@@ -1598,34 +1598,34 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>9781119560822</t>
+          <t>9781119560821</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>BC9781119560822-01</t>
+          <t>BC9781119560821-01</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-0822-1</t>
+          <t>Kệ GEN-0821-1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>9781119560822</t>
+          <t>9781119560821</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>BC9781119560822-02</t>
+          <t>BC9781119560821-02</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Kệ GEN-0822-2</t>
+          <t>Kệ GEN-0821-2</t>
         </is>
       </c>
     </row>

</xml_diff>